<commit_message>
Start counting directly from verified Excel import
</commit_message>
<xml_diff>
--- a/warehouse-demo-sample.xlsx
+++ b/warehouse-demo-sample.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="盤點明細" sheetId="1" r:id="R00896e3345784102"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="盤點明細" sheetId="1" r:id="R9d79af05ce0c4cec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -266,6 +266,7 @@
     <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="22" customHeight="1">
@@ -284,6 +285,9 @@
       <x:c r="E1" s="3" t="str">
         <x:v>文中數量</x:v>
       </x:c>
+      <x:c r="F1" s="3" t="str">
+        <x:v>單位</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="1" t="str">
@@ -301,6 +305,9 @@
       <x:c r="E2" s="1" t="n">
         <x:v>12</x:v>
       </x:c>
+      <x:c r="F2" s="1" t="str">
+        <x:v>件</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="1" t="str">
@@ -318,6 +325,9 @@
       <x:c r="E3" s="1" t="n">
         <x:v>7</x:v>
       </x:c>
+      <x:c r="F3" s="1" t="str">
+        <x:v>件</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="1" t="str">
@@ -335,6 +345,9 @@
       <x:c r="E4" s="1" t="n">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F4" s="1" t="str">
+        <x:v>件</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
       <x:c r="A5" s="1" t="str">
@@ -351,6 +364,9 @@
       </x:c>
       <x:c r="E5" s="1" t="n">
         <x:v>20</x:v>
+      </x:c>
+      <x:c r="F5" s="1" t="str">
+        <x:v>件</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>